<commit_message>
chore(data-release): publish site data 2026-09-19 18:12:35 UTC
</commit_message>
<xml_diff>
--- a/countries/de/2020-2025.xlsx
+++ b/countries/de/2020-2025.xlsx
@@ -48706,13 +48706,13 @@
         </is>
       </c>
       <c r="N246" t="n">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="O246" t="n">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="R246" t="n">
-        <v>0.6552797285101162</v>
+        <v>0.6564689839157607</v>
       </c>
       <c r="S246" t="inlineStr">
         <is>
@@ -48865,10 +48865,10 @@
         </is>
       </c>
       <c r="N247" t="n">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="O247" t="n">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="U247" t="inlineStr">
         <is>
@@ -61282,13 +61282,13 @@
         </is>
       </c>
       <c r="N310" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="O310" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="R310" t="n">
-        <v>0.2365513714887778</v>
+        <v>0.2377341283462217</v>
       </c>
       <c r="S310" t="inlineStr">
         <is>
@@ -61441,10 +61441,10 @@
         </is>
       </c>
       <c r="N311" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="O311" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="U311" t="inlineStr">
         <is>
@@ -72679,13 +72679,13 @@
         </is>
       </c>
       <c r="N368" t="n">
-        <v>994</v>
+        <v>1005</v>
       </c>
       <c r="O368" t="n">
-        <v>994</v>
+        <v>1005</v>
       </c>
       <c r="R368" t="n">
-        <v>1.175604545175751</v>
+        <v>1.188614253422162</v>
       </c>
       <c r="S368" t="inlineStr">
         <is>
@@ -72838,10 +72838,10 @@
         </is>
       </c>
       <c r="N369" t="n">
-        <v>994</v>
+        <v>1005</v>
       </c>
       <c r="O369" t="n">
-        <v>994</v>
+        <v>1005</v>
       </c>
       <c r="U369" t="inlineStr">
         <is>
@@ -75037,13 +75037,13 @@
         </is>
       </c>
       <c r="N380" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O380" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="R380" t="n">
-        <v>0.06386584048238483</v>
+        <v>0.06504854123205864</v>
       </c>
       <c r="S380" t="inlineStr">
         <is>
@@ -75196,10 +75196,10 @@
         </is>
       </c>
       <c r="N381" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O381" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="U381" t="inlineStr">
         <is>
@@ -77002,13 +77002,13 @@
         </is>
       </c>
       <c r="N390" t="n">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="O390" t="n">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="R390" t="n">
-        <v>0.2152515364406304</v>
+        <v>0.2270785439373683</v>
       </c>
       <c r="S390" t="inlineStr">
         <is>
@@ -77161,10 +77161,10 @@
         </is>
       </c>
       <c r="N391" t="n">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="O391" t="n">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="U391" t="inlineStr">
         <is>
@@ -78574,13 +78574,13 @@
         </is>
       </c>
       <c r="N398" t="n">
-        <v>45989</v>
+        <v>46112</v>
       </c>
       <c r="O398" t="n">
-        <v>45989</v>
+        <v>46112</v>
       </c>
       <c r="R398" t="n">
-        <v>54.39122477674808</v>
+        <v>54.53669696895796</v>
       </c>
       <c r="S398" t="inlineStr">
         <is>
@@ -78733,10 +78733,10 @@
         </is>
       </c>
       <c r="N399" t="n">
-        <v>45989</v>
+        <v>46112</v>
       </c>
       <c r="O399" t="n">
-        <v>45989</v>
+        <v>46112</v>
       </c>
       <c r="U399" t="inlineStr">
         <is>
@@ -79360,13 +79360,13 @@
         </is>
       </c>
       <c r="N402" t="n">
-        <v>2210</v>
+        <v>2213</v>
       </c>
       <c r="O402" t="n">
-        <v>2210</v>
+        <v>2213</v>
       </c>
       <c r="R402" t="n">
-        <v>2.613768656779083</v>
+        <v>2.617316759028105</v>
       </c>
       <c r="S402" t="inlineStr">
         <is>
@@ -79519,10 +79519,10 @@
         </is>
       </c>
       <c r="N403" t="n">
-        <v>2210</v>
+        <v>2213</v>
       </c>
       <c r="O403" t="n">
-        <v>2210</v>
+        <v>2213</v>
       </c>
       <c r="U403" t="inlineStr">
         <is>
@@ -80146,13 +80146,13 @@
         </is>
       </c>
       <c r="N406" t="n">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="O406" t="n">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="R406" t="n">
-        <v>0.7640246842892705</v>
+        <v>0.7663900857886181</v>
       </c>
       <c r="S406" t="inlineStr">
         <is>
@@ -80305,10 +80305,10 @@
         </is>
       </c>
       <c r="N407" t="n">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="O407" t="n">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="U407" t="inlineStr">
         <is>
@@ -80932,13 +80932,13 @@
         </is>
       </c>
       <c r="N410" t="n">
-        <v>12316</v>
+        <v>12356</v>
       </c>
       <c r="O410" t="n">
-        <v>12316</v>
+        <v>12356</v>
       </c>
       <c r="R410" t="n">
-        <v>14.56614243298244</v>
+        <v>14.61345046296939</v>
       </c>
       <c r="S410" t="inlineStr">
         <is>
@@ -81091,10 +81091,10 @@
         </is>
       </c>
       <c r="N411" t="n">
-        <v>12316</v>
+        <v>12356</v>
       </c>
       <c r="O411" t="n">
-        <v>12316</v>
+        <v>12356</v>
       </c>
       <c r="U411" t="inlineStr">
         <is>
@@ -81325,13 +81325,13 @@
         </is>
       </c>
       <c r="N412" t="n">
-        <v>4580</v>
+        <v>4591</v>
       </c>
       <c r="O412" t="n">
-        <v>4580</v>
+        <v>4591</v>
       </c>
       <c r="R412" t="n">
-        <v>5.416769433505974</v>
+        <v>5.429779141752386</v>
       </c>
       <c r="S412" t="inlineStr">
         <is>
@@ -81484,10 +81484,10 @@
         </is>
       </c>
       <c r="N413" t="n">
-        <v>4580</v>
+        <v>4591</v>
       </c>
       <c r="O413" t="n">
-        <v>4580</v>
+        <v>4591</v>
       </c>
       <c r="U413" t="inlineStr">
         <is>
@@ -84440,17 +84440,17 @@
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t>D017</t>
+          <t>D007</t>
         </is>
       </c>
       <c r="I428" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>Hepatitis A</t>
         </is>
       </c>
       <c r="J428" t="inlineStr">
         <is>
-          <t>麻疹</t>
+          <t>甲型肝炎</t>
         </is>
       </c>
       <c r="K428" t="inlineStr">
@@ -84469,13 +84469,13 @@
         </is>
       </c>
       <c r="N428" t="n">
-        <v>241</v>
+        <v>1134</v>
       </c>
       <c r="O428" t="n">
-        <v>241</v>
+        <v>1134</v>
       </c>
       <c r="R428" t="n">
-        <v>0.2866485714502697</v>
+        <v>1.348794522923676</v>
       </c>
       <c r="S428" t="inlineStr">
         <is>
@@ -84484,7 +84484,7 @@
       </c>
       <c r="U428" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_MEAS_ANNUAL</t>
+          <t>SER_DE_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="AA428" t="inlineStr">
@@ -84509,7 +84509,7 @@
       </c>
       <c r="AS428" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_MEAS_ANNUAL</t>
+          <t>SER_DE_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="AT428" t="n">
@@ -84599,17 +84599,17 @@
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t>D017</t>
+          <t>D007</t>
         </is>
       </c>
       <c r="I429" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>Hepatitis A</t>
         </is>
       </c>
       <c r="J429" t="inlineStr">
         <is>
-          <t>麻疹</t>
+          <t>甲型肝炎</t>
         </is>
       </c>
       <c r="K429" t="inlineStr">
@@ -84628,19 +84628,19 @@
         </is>
       </c>
       <c r="N429" t="n">
-        <v>241</v>
+        <v>1134</v>
       </c>
       <c r="O429" t="n">
-        <v>241</v>
+        <v>1134</v>
       </c>
       <c r="U429" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_MEAS_ANNUAL</t>
+          <t>SER_DE_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="V429" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_MEAS_ANNUAL</t>
+          <t>SER_DE_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="W429" t="inlineStr">
@@ -84650,7 +84650,7 @@
       </c>
       <c r="X429" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>Hepatitis A</t>
         </is>
       </c>
       <c r="Y429" t="inlineStr">
@@ -84743,7 +84743,7 @@
       </c>
       <c r="AS429" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_MEAS_ANNUAL</t>
+          <t>SER_DE_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="AT429" t="n">
@@ -84833,22 +84833,22 @@
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t>D029</t>
+          <t>D017</t>
         </is>
       </c>
       <c r="I430" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="J430" t="inlineStr">
         <is>
-          <t>白喉</t>
+          <t>麻疹</t>
         </is>
       </c>
       <c r="K430" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L430" t="inlineStr">
@@ -84862,13 +84862,13 @@
         </is>
       </c>
       <c r="N430" t="n">
-        <v>46</v>
+        <v>241</v>
       </c>
       <c r="O430" t="n">
-        <v>46</v>
+        <v>241</v>
       </c>
       <c r="R430" t="n">
-        <v>0.05471300533905563</v>
+        <v>0.2866485714502697</v>
       </c>
       <c r="S430" t="inlineStr">
         <is>
@@ -84877,7 +84877,7 @@
       </c>
       <c r="U430" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_DIPH_ANNUAL</t>
+          <t>SER_DE_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="AA430" t="inlineStr">
@@ -84902,7 +84902,7 @@
       </c>
       <c r="AS430" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_DIPH_ANNUAL</t>
+          <t>SER_DE_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="AT430" t="n">
@@ -84992,22 +84992,22 @@
       </c>
       <c r="H431" t="inlineStr">
         <is>
-          <t>D029</t>
+          <t>D017</t>
         </is>
       </c>
       <c r="I431" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="J431" t="inlineStr">
         <is>
-          <t>白喉</t>
+          <t>麻疹</t>
         </is>
       </c>
       <c r="K431" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L431" t="inlineStr">
@@ -85021,19 +85021,19 @@
         </is>
       </c>
       <c r="N431" t="n">
-        <v>46</v>
+        <v>241</v>
       </c>
       <c r="O431" t="n">
-        <v>46</v>
+        <v>241</v>
       </c>
       <c r="U431" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_DIPH_ANNUAL</t>
+          <t>SER_DE_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="V431" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_DIPH_ANNUAL</t>
+          <t>SER_DE_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="W431" t="inlineStr">
@@ -85043,7 +85043,7 @@
       </c>
       <c r="X431" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="Y431" t="inlineStr">
@@ -85136,7 +85136,7 @@
       </c>
       <c r="AS431" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_DIPH_ANNUAL</t>
+          <t>SER_DE_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="AT431" t="n">
@@ -85226,22 +85226,22 @@
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t>D040</t>
+          <t>D029</t>
         </is>
       </c>
       <c r="I432" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="J432" t="inlineStr">
         <is>
-          <t>风疹</t>
+          <t>白喉</t>
         </is>
       </c>
       <c r="K432" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L432" t="inlineStr">
@@ -85255,13 +85255,13 @@
         </is>
       </c>
       <c r="N432" t="n">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="O432" t="n">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="R432" t="n">
-        <v>0.009515305276357501</v>
+        <v>0.05471300533905563</v>
       </c>
       <c r="S432" t="inlineStr">
         <is>
@@ -85270,7 +85270,7 @@
       </c>
       <c r="U432" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_RUBE_ANNUAL</t>
+          <t>SER_DE_ECDC_DIPH_ANNUAL</t>
         </is>
       </c>
       <c r="AA432" t="inlineStr">
@@ -85295,7 +85295,7 @@
       </c>
       <c r="AS432" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_RUBE_ANNUAL</t>
+          <t>SER_DE_ECDC_DIPH_ANNUAL</t>
         </is>
       </c>
       <c r="AT432" t="n">
@@ -85385,22 +85385,22 @@
       </c>
       <c r="H433" t="inlineStr">
         <is>
-          <t>D040</t>
+          <t>D029</t>
         </is>
       </c>
       <c r="I433" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="J433" t="inlineStr">
         <is>
-          <t>风疹</t>
+          <t>白喉</t>
         </is>
       </c>
       <c r="K433" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L433" t="inlineStr">
@@ -85414,19 +85414,19 @@
         </is>
       </c>
       <c r="N433" t="n">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="O433" t="n">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="U433" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_RUBE_ANNUAL</t>
+          <t>SER_DE_ECDC_DIPH_ANNUAL</t>
         </is>
       </c>
       <c r="V433" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_RUBE_ANNUAL</t>
+          <t>SER_DE_ECDC_DIPH_ANNUAL</t>
         </is>
       </c>
       <c r="W433" t="inlineStr">
@@ -85436,7 +85436,7 @@
       </c>
       <c r="X433" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="Y433" t="inlineStr">
@@ -85529,7 +85529,7 @@
       </c>
       <c r="AS433" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_RUBE_ANNUAL</t>
+          <t>SER_DE_ECDC_DIPH_ANNUAL</t>
         </is>
       </c>
       <c r="AT433" t="n">
@@ -85619,17 +85619,17 @@
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t>D107</t>
+          <t>D032</t>
         </is>
       </c>
       <c r="I434" t="inlineStr">
         <is>
-          <t>Legionellosis</t>
+          <t>Brucellosis</t>
         </is>
       </c>
       <c r="J434" t="inlineStr">
         <is>
-          <t>军团菌病</t>
+          <t>布鲁氏菌病</t>
         </is>
       </c>
       <c r="K434" t="inlineStr">
@@ -85648,13 +85648,13 @@
         </is>
       </c>
       <c r="N434" t="n">
-        <v>2229</v>
+        <v>53</v>
       </c>
       <c r="O434" t="n">
-        <v>2229</v>
+        <v>53</v>
       </c>
       <c r="R434" t="n">
-        <v>2.651201932625109</v>
+        <v>0.06303889745586845</v>
       </c>
       <c r="S434" t="inlineStr">
         <is>
@@ -85663,7 +85663,7 @@
       </c>
       <c r="U434" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_LEGI_ANNUAL</t>
+          <t>SER_DE_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="AA434" t="inlineStr">
@@ -85688,7 +85688,7 @@
       </c>
       <c r="AS434" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_LEGI_ANNUAL</t>
+          <t>SER_DE_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="AT434" t="n">
@@ -85778,17 +85778,17 @@
       </c>
       <c r="H435" t="inlineStr">
         <is>
-          <t>D107</t>
+          <t>D032</t>
         </is>
       </c>
       <c r="I435" t="inlineStr">
         <is>
-          <t>Legionellosis</t>
+          <t>Brucellosis</t>
         </is>
       </c>
       <c r="J435" t="inlineStr">
         <is>
-          <t>军团菌病</t>
+          <t>布鲁氏菌病</t>
         </is>
       </c>
       <c r="K435" t="inlineStr">
@@ -85807,19 +85807,19 @@
         </is>
       </c>
       <c r="N435" t="n">
-        <v>2229</v>
+        <v>53</v>
       </c>
       <c r="O435" t="n">
-        <v>2229</v>
+        <v>53</v>
       </c>
       <c r="U435" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_LEGI_ANNUAL</t>
+          <t>SER_DE_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="V435" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_LEGI_ANNUAL</t>
+          <t>SER_DE_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="W435" t="inlineStr">
@@ -85829,7 +85829,7 @@
       </c>
       <c r="X435" t="inlineStr">
         <is>
-          <t>Legionnaires' disease</t>
+          <t>Brucellosis</t>
         </is>
       </c>
       <c r="Y435" t="inlineStr">
@@ -85922,7 +85922,7 @@
       </c>
       <c r="AS435" t="inlineStr">
         <is>
-          <t>SER_DE_ECDC_LEGI_ANNUAL</t>
+          <t>SER_DE_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="AT435" t="n">
@@ -85969,6 +85969,3936 @@
         </is>
       </c>
       <c r="BC435" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>D040</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>风疹</t>
+        </is>
+      </c>
+      <c r="K436" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L436" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M436" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N436" t="n">
+        <v>8</v>
+      </c>
+      <c r="O436" t="n">
+        <v>8</v>
+      </c>
+      <c r="R436" t="n">
+        <v>0.009515305276357501</v>
+      </c>
+      <c r="S436" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U436" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA436" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO436" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP436" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ436" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS436" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT436" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU436" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV436" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW436" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX436" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY436" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ436" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA436" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB436" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC436" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>D040</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>风疹</t>
+        </is>
+      </c>
+      <c r="K437" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N437" t="n">
+        <v>8</v>
+      </c>
+      <c r="O437" t="n">
+        <v>8</v>
+      </c>
+      <c r="U437" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V437" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W437" t="inlineStr">
+        <is>
+          <t>SRC_DE_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X437" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="Y437" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z437" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA437" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB437" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC437" t="inlineStr">
+        <is>
+          <t>country:DE:national</t>
+        </is>
+      </c>
+      <c r="AD437" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE437" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF437" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG437" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH437" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI437" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ437" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK437" t="inlineStr">
+        <is>
+          <t>Germany annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM437" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN437" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO437" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP437" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ437" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS437" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT437" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU437" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV437" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW437" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX437" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY437" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ437" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA437" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB437" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC437" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>D045</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>Echinococcosis</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>包虫病</t>
+        </is>
+      </c>
+      <c r="K438" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N438" t="n">
+        <v>159</v>
+      </c>
+      <c r="O438" t="n">
+        <v>159</v>
+      </c>
+      <c r="R438" t="n">
+        <v>0.1891166923676053</v>
+      </c>
+      <c r="S438" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U438" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA438" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO438" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP438" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ438" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS438" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT438" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU438" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV438" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW438" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX438" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY438" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ438" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA438" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB438" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC438" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>D045</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>Echinococcosis</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>包虫病</t>
+        </is>
+      </c>
+      <c r="K439" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L439" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M439" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N439" t="n">
+        <v>159</v>
+      </c>
+      <c r="O439" t="n">
+        <v>159</v>
+      </c>
+      <c r="U439" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V439" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W439" t="inlineStr">
+        <is>
+          <t>SRC_DE_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X439" t="inlineStr">
+        <is>
+          <t>Echinococcosis</t>
+        </is>
+      </c>
+      <c r="Y439" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z439" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA439" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB439" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC439" t="inlineStr">
+        <is>
+          <t>country:DE:national</t>
+        </is>
+      </c>
+      <c r="AD439" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE439" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF439" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG439" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH439" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI439" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ439" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK439" t="inlineStr">
+        <is>
+          <t>Germany annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM439" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN439" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO439" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP439" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ439" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS439" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT439" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU439" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV439" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW439" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX439" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY439" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ439" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA439" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB439" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC439" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>D085</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>Toxoplasmosis</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>弓形体病</t>
+        </is>
+      </c>
+      <c r="K440" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L440" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M440" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N440" t="n">
+        <v>2</v>
+      </c>
+      <c r="O440" t="n">
+        <v>2</v>
+      </c>
+      <c r="R440" t="n">
+        <v>0.002378826319089375</v>
+      </c>
+      <c r="S440" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U440" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_TOXO_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA440" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO440" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP440" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ440" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS440" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_TOXO_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT440" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU440" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV440" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW440" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX440" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY440" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ440" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA440" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB440" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC440" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>D085</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>Toxoplasmosis</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>弓形体病</t>
+        </is>
+      </c>
+      <c r="K441" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L441" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M441" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N441" t="n">
+        <v>2</v>
+      </c>
+      <c r="O441" t="n">
+        <v>2</v>
+      </c>
+      <c r="U441" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_TOXO_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V441" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_TOXO_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W441" t="inlineStr">
+        <is>
+          <t>SRC_DE_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X441" t="inlineStr">
+        <is>
+          <t>Toxoplasmosis, congenital</t>
+        </is>
+      </c>
+      <c r="Y441" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z441" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA441" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB441" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC441" t="inlineStr">
+        <is>
+          <t>country:DE:national</t>
+        </is>
+      </c>
+      <c r="AD441" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE441" t="inlineStr">
+        <is>
+          <t>narrower</t>
+        </is>
+      </c>
+      <c r="AF441" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG441" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH441" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI441" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ441" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK441" t="inlineStr">
+        <is>
+          <t>Germany annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM441" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN441" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO441" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP441" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ441" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS441" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_TOXO_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT441" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU441" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV441" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW441" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX441" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY441" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ441" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA441" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB441" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC441" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>D092</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>Campylobacteriosis</t>
+        </is>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>弯曲杆菌病</t>
+        </is>
+      </c>
+      <c r="K442" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M442" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N442" t="n">
+        <v>49933</v>
+      </c>
+      <c r="O442" t="n">
+        <v>49933</v>
+      </c>
+      <c r="R442" t="n">
+        <v>59.39096729554488</v>
+      </c>
+      <c r="S442" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U442" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA442" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO442" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP442" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ442" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS442" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT442" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU442" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV442" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW442" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX442" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY442" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ442" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA442" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB442" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC442" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>D092</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>Campylobacteriosis</t>
+        </is>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>弯曲杆菌病</t>
+        </is>
+      </c>
+      <c r="K443" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M443" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N443" t="n">
+        <v>49933</v>
+      </c>
+      <c r="O443" t="n">
+        <v>49933</v>
+      </c>
+      <c r="U443" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V443" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W443" t="inlineStr">
+        <is>
+          <t>SRC_DE_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X443" t="inlineStr">
+        <is>
+          <t>Campylobacteriosis</t>
+        </is>
+      </c>
+      <c r="Y443" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z443" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA443" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB443" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC443" t="inlineStr">
+        <is>
+          <t>country:DE:national</t>
+        </is>
+      </c>
+      <c r="AD443" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE443" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF443" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG443" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH443" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI443" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ443" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK443" t="inlineStr">
+        <is>
+          <t>Germany annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM443" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN443" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO443" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP443" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ443" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS443" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT443" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU443" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV443" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW443" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX443" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY443" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ443" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA443" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB443" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC443" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>D105</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>Shigellosis</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>志贺菌病</t>
+        </is>
+      </c>
+      <c r="K444" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M444" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N444" t="n">
+        <v>3331</v>
+      </c>
+      <c r="O444" t="n">
+        <v>3331</v>
+      </c>
+      <c r="R444" t="n">
+        <v>3.961935234443354</v>
+      </c>
+      <c r="S444" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U444" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA444" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO444" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP444" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ444" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS444" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT444" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU444" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV444" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW444" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX444" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY444" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ444" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA444" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB444" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC444" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>D105</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>Shigellosis</t>
+        </is>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>志贺菌病</t>
+        </is>
+      </c>
+      <c r="K445" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L445" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M445" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N445" t="n">
+        <v>3331</v>
+      </c>
+      <c r="O445" t="n">
+        <v>3331</v>
+      </c>
+      <c r="U445" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V445" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W445" t="inlineStr">
+        <is>
+          <t>SRC_DE_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X445" t="inlineStr">
+        <is>
+          <t>Shigellosis</t>
+        </is>
+      </c>
+      <c r="Y445" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z445" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA445" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB445" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC445" t="inlineStr">
+        <is>
+          <t>country:DE:national</t>
+        </is>
+      </c>
+      <c r="AD445" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE445" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF445" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG445" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH445" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI445" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ445" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK445" t="inlineStr">
+        <is>
+          <t>Germany annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM445" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN445" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO445" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP445" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ445" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS445" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT445" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU445" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV445" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW445" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX445" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY445" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ445" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA445" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB445" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC445" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>D107</t>
+        </is>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>Legionellosis</t>
+        </is>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>军团菌病</t>
+        </is>
+      </c>
+      <c r="K446" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L446" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M446" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N446" t="n">
+        <v>2229</v>
+      </c>
+      <c r="O446" t="n">
+        <v>2229</v>
+      </c>
+      <c r="R446" t="n">
+        <v>2.651201932625109</v>
+      </c>
+      <c r="S446" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U446" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA446" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO446" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP446" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ446" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS446" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT446" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU446" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV446" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW446" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX446" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY446" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ446" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA446" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB446" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC446" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>D107</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>Legionellosis</t>
+        </is>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>军团菌病</t>
+        </is>
+      </c>
+      <c r="K447" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L447" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M447" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N447" t="n">
+        <v>2229</v>
+      </c>
+      <c r="O447" t="n">
+        <v>2229</v>
+      </c>
+      <c r="U447" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V447" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W447" t="inlineStr">
+        <is>
+          <t>SRC_DE_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X447" t="inlineStr">
+        <is>
+          <t>Legionnaires' disease</t>
+        </is>
+      </c>
+      <c r="Y447" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z447" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA447" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB447" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC447" t="inlineStr">
+        <is>
+          <t>country:DE:national</t>
+        </is>
+      </c>
+      <c r="AD447" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE447" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF447" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG447" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH447" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI447" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ447" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK447" t="inlineStr">
+        <is>
+          <t>Germany annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM447" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN447" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO447" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP447" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ447" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS447" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT447" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU447" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV447" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW447" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX447" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY447" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ447" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA447" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB447" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC447" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>D108</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>Listeriosis</t>
+        </is>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>李斯特菌病</t>
+        </is>
+      </c>
+      <c r="K448" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M448" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N448" t="n">
+        <v>595</v>
+      </c>
+      <c r="O448" t="n">
+        <v>595</v>
+      </c>
+      <c r="R448" t="n">
+        <v>0.7077008299290891</v>
+      </c>
+      <c r="S448" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U448" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA448" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO448" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP448" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ448" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS448" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT448" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU448" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV448" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW448" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX448" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY448" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ448" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA448" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB448" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC448" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>D108</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>Listeriosis</t>
+        </is>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>李斯特菌病</t>
+        </is>
+      </c>
+      <c r="K449" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M449" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N449" t="n">
+        <v>595</v>
+      </c>
+      <c r="O449" t="n">
+        <v>595</v>
+      </c>
+      <c r="U449" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V449" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W449" t="inlineStr">
+        <is>
+          <t>SRC_DE_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X449" t="inlineStr">
+        <is>
+          <t>Listeriosis</t>
+        </is>
+      </c>
+      <c r="Y449" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z449" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA449" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB449" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC449" t="inlineStr">
+        <is>
+          <t>country:DE:national</t>
+        </is>
+      </c>
+      <c r="AD449" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE449" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF449" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG449" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH449" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI449" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ449" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK449" t="inlineStr">
+        <is>
+          <t>Germany annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM449" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN449" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO449" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP449" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ449" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS449" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT449" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU449" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV449" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW449" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX449" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY449" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ449" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA449" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB449" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC449" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>D114</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>Salmonellosis</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>沙门氏菌病</t>
+        </is>
+      </c>
+      <c r="K450" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M450" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N450" t="n">
+        <v>10578</v>
+      </c>
+      <c r="O450" t="n">
+        <v>10578</v>
+      </c>
+      <c r="R450" t="n">
+        <v>12.5816124016637</v>
+      </c>
+      <c r="S450" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U450" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA450" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO450" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP450" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ450" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS450" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT450" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU450" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV450" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW450" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX450" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY450" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ450" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA450" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB450" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC450" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>D114</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>Salmonellosis</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>沙门氏菌病</t>
+        </is>
+      </c>
+      <c r="K451" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M451" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N451" t="n">
+        <v>10578</v>
+      </c>
+      <c r="O451" t="n">
+        <v>10578</v>
+      </c>
+      <c r="U451" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V451" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W451" t="inlineStr">
+        <is>
+          <t>SRC_DE_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X451" t="inlineStr">
+        <is>
+          <t>Salmonellosis</t>
+        </is>
+      </c>
+      <c r="Y451" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z451" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA451" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB451" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC451" t="inlineStr">
+        <is>
+          <t>country:DE:national</t>
+        </is>
+      </c>
+      <c r="AD451" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE451" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF451" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG451" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH451" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI451" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ451" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK451" t="inlineStr">
+        <is>
+          <t>Germany annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM451" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN451" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO451" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP451" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ451" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS451" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT451" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU451" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV451" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW451" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX451" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY451" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ451" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA451" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB451" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC451" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>D115</t>
+        </is>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>Shiga toxin-producing Escherichia coli infection</t>
+        </is>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>产志贺毒素大肠杆菌感染</t>
+        </is>
+      </c>
+      <c r="K452" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M452" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N452" t="n">
+        <v>6658</v>
+      </c>
+      <c r="O452" t="n">
+        <v>6658</v>
+      </c>
+      <c r="R452" t="n">
+        <v>7.91911281624853</v>
+      </c>
+      <c r="S452" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U452" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA452" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO452" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP452" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ452" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS452" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT452" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU452" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV452" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW452" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX452" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY452" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ452" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA452" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB452" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC452" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>D115</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>Shiga toxin-producing Escherichia coli infection</t>
+        </is>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>产志贺毒素大肠杆菌感染</t>
+        </is>
+      </c>
+      <c r="K453" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L453" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M453" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N453" t="n">
+        <v>6658</v>
+      </c>
+      <c r="O453" t="n">
+        <v>6658</v>
+      </c>
+      <c r="U453" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V453" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W453" t="inlineStr">
+        <is>
+          <t>SRC_DE_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X453" t="inlineStr">
+        <is>
+          <t>STEC/VTEC infection</t>
+        </is>
+      </c>
+      <c r="Y453" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z453" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA453" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB453" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC453" t="inlineStr">
+        <is>
+          <t>country:DE:national</t>
+        </is>
+      </c>
+      <c r="AD453" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE453" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF453" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG453" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH453" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI453" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ453" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK453" t="inlineStr">
+        <is>
+          <t>Germany annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM453" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN453" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO453" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP453" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ453" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS453" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT453" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU453" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV453" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW453" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX453" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY453" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ453" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA453" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB453" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC453" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>D122</t>
+        </is>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>Trichinellosis</t>
+        </is>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>旋毛虫病</t>
+        </is>
+      </c>
+      <c r="K454" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L454" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M454" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N454" t="n">
+        <v>2</v>
+      </c>
+      <c r="O454" t="n">
+        <v>2</v>
+      </c>
+      <c r="R454" t="n">
+        <v>0.002378826319089375</v>
+      </c>
+      <c r="S454" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U454" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA454" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO454" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP454" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ454" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS454" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT454" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU454" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV454" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW454" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX454" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY454" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ454" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA454" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB454" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC454" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>D122</t>
+        </is>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>Trichinellosis</t>
+        </is>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>旋毛虫病</t>
+        </is>
+      </c>
+      <c r="K455" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L455" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M455" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N455" t="n">
+        <v>2</v>
+      </c>
+      <c r="O455" t="n">
+        <v>2</v>
+      </c>
+      <c r="U455" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V455" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W455" t="inlineStr">
+        <is>
+          <t>SRC_DE_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X455" t="inlineStr">
+        <is>
+          <t>Trichinellosis</t>
+        </is>
+      </c>
+      <c r="Y455" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z455" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA455" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB455" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC455" t="inlineStr">
+        <is>
+          <t>country:DE:national</t>
+        </is>
+      </c>
+      <c r="AD455" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE455" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF455" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG455" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH455" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI455" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ455" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK455" t="inlineStr">
+        <is>
+          <t>Germany annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM455" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN455" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO455" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP455" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ455" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS455" t="inlineStr">
+        <is>
+          <t>SER_DE_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT455" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU455" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV455" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW455" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX455" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY455" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ455" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA455" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB455" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC455" t="inlineStr">
         <is>
           <t>official_webforms_csv_export</t>
         </is>
@@ -86090,7 +90020,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>217</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10">
@@ -86100,7 +90030,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>434</v>
+        <v>454</v>
       </c>
     </row>
     <row r="11">
@@ -86120,7 +90050,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>217</v>
+        <v>227</v>
       </c>
     </row>
     <row r="13">
@@ -86152,7 +90082,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>492837</v>
+        <v>565485</v>
       </c>
     </row>
     <row r="16">

</xml_diff>